<commit_message>
Refresh published budget figures
</commit_message>
<xml_diff>
--- a/Бюджет Октоберфест.xlsx
+++ b/Бюджет Октоберфест.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Desktop\Новая папка\Заполнено_в работу\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B914BD-7C80-43FC-AF6C-8D88DDBB9F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{676D059A-E334-4F4E-B3BD-71A6E777574B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Октоберфест" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t>Средний чек</t>
   </si>
@@ -80,52 +80,64 @@
     <t>Повара</t>
   </si>
   <si>
+    <t>Клининг</t>
+  </si>
+  <si>
+    <t>Официанты</t>
+  </si>
+  <si>
+    <t>Бармены</t>
+  </si>
+  <si>
+    <t>Ивенты ФОТ</t>
+  </si>
+  <si>
+    <t>час</t>
+  </si>
+  <si>
+    <t>Призовой фонд</t>
+  </si>
+  <si>
+    <t>Изготовление и поставка рекламного баннера</t>
+  </si>
+  <si>
+    <t>Аниматоры</t>
+  </si>
+  <si>
+    <t>Ведущий (13 часов)</t>
+  </si>
+  <si>
+    <t>Аниматоры (по 5 часов)</t>
+  </si>
+  <si>
+    <t>Диджей (3 часа)</t>
+  </si>
+  <si>
+    <t>Мастер классы (аниматоры 6 часов)</t>
+  </si>
+  <si>
+    <t>Мастер классы (расходники на 2 дня)</t>
+  </si>
+  <si>
+    <t>Аренда оборудования (для ведущего и диджея)</t>
+  </si>
+  <si>
+    <t>день</t>
+  </si>
+  <si>
+    <t>Оборудование ФУД</t>
+  </si>
+  <si>
+    <t>Стоимость гриля (за 3 шт)</t>
+  </si>
+  <si>
+    <t>налоги на ФОТ ФУД (*1,46)</t>
+  </si>
+  <si>
     <t>смена</t>
   </si>
   <si>
-    <t>Клининг</t>
-  </si>
-  <si>
-    <t>Официанты</t>
-  </si>
-  <si>
-    <t>Бармены</t>
-  </si>
-  <si>
-    <t>Ивенты ФОТ</t>
-  </si>
-  <si>
-    <t>Ведущий</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Аниматоры </t>
-  </si>
-  <si>
-    <t>час</t>
-  </si>
-  <si>
-    <t>с НДС 6%</t>
-  </si>
-  <si>
-    <t>Диджей</t>
-  </si>
-  <si>
-    <t>Мастер классы (аниматоры)</t>
-  </si>
-  <si>
-    <t>Мастер классы (расходники)</t>
-  </si>
-  <si>
-    <t>Призовой фонд</t>
-  </si>
-  <si>
-    <t>Оборудование для Фуд</t>
-  </si>
-  <si>
-    <t>Аренда оборудования для Анимации</t>
-  </si>
-  <si>
-    <t>Изготовление и поставка рекламного баннера</t>
+    <t>Покупаем один раз и используем на всех фестивалях</t>
   </si>
 </sst>
 </file>
@@ -135,7 +147,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;₽&quot;_-;\-* #,##0.00\ &quot;₽&quot;_-;_-* &quot;-&quot;??\ &quot;₽&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,31 +184,7 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
@@ -205,13 +193,29 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -238,13 +242,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -343,15 +341,13 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -360,12 +356,8 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -392,39 +384,26 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="3" fillId="4" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="5" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="3" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="4" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="5" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="6" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Денежный" xfId="1" builtinId="4"/>
@@ -741,390 +720,448 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B06DD981-710B-49F4-BD8B-F9607C12061A}">
-  <dimension ref="B2:G39"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:G42"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="38.90625" customWidth="1"/>
-    <col min="3" max="3" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12.26953125" customWidth="1"/>
-    <col min="6" max="6" width="19.08984375" customWidth="1"/>
-    <col min="7" max="7" width="8.984375E-2" customWidth="1"/>
+    <col min="2" max="2" width="42.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.7265625" customWidth="1"/>
+    <col min="4" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="5" width="12.26953125" customWidth="1"/>
+    <col min="6" max="6" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="37">
+      <c r="C2" s="19">
         <v>2500</v>
       </c>
     </row>
-    <row r="3" spans="2:6" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="38">
+      <c r="C3">
         <v>5000</v>
       </c>
     </row>
-    <row r="4" spans="2:6" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="39">
+      <c r="C4" s="20">
         <v>0.23</v>
       </c>
-    </row>
-    <row r="5" spans="2:6" outlineLevel="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="20">
+        <v>0.46</v>
+      </c>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="38">
+      <c r="C6">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="37">
+      <c r="C8" s="19">
         <v>20000</v>
       </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="C7" s="1"/>
-    </row>
-    <row r="11" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="3" t="s">
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+    </row>
+    <row r="13" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F13" s="21"/>
+    </row>
+    <row r="14" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="5">
-        <f>F15-F20</f>
-        <v>6829531.9138297876</v>
-      </c>
-    </row>
-    <row r="13" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="23"/>
-    </row>
-    <row r="14" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="3">
+        <f>F17-F22</f>
+        <v>6718671.9148936169</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="23"/>
+    </row>
+    <row r="16" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="8">
-        <f>F15</f>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="6">
+        <f>F17</f>
         <v>12500000</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B15" s="9" t="s">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B17" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="10">
-        <f>SUM(F16:F18)</f>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="8">
+        <f>SUM(F18:F20)</f>
         <v>12500000</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B16" s="11" t="s">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B18" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="12">
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="10">
         <f>C2*C3</f>
         <v>12500000</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="19" spans="2:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="13" t="s">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+    </row>
+    <row r="21" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B21" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="21">
-        <f>F20</f>
-        <v>5670468.0861702124</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B20" s="15" t="s">
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="25">
+        <f>F22</f>
+        <v>5781328.0851063831</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B22" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="16">
-        <f>F21+F22+F23+F24+F36+F37+F29+F34+F35</f>
-        <v>5670468.0861702124</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B21" s="25" t="s">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="14">
+        <f>F23+F24+F25+F26+F38+F40+F31+F36+F37</f>
+        <v>5781328.0851063831</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B23" s="26" t="s">
         <v>11</v>
-      </c>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="28">
-        <v>400000</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="36" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="28">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B23" s="27" t="s">
-        <v>8</v>
       </c>
       <c r="C23" s="27"/>
       <c r="D23" s="27"/>
       <c r="E23" s="27"/>
-      <c r="F23" s="29">
-        <f>C2*C3*C4</f>
-        <v>2875000</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B24" s="27" t="s">
-        <v>12</v>
+      <c r="F23" s="28">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B24" s="26" t="s">
+        <v>20</v>
       </c>
       <c r="C24" s="27"/>
       <c r="D24" s="27"/>
       <c r="E24" s="27"/>
-      <c r="F24" s="30">
-        <f>SUM(F25:F28)*C5</f>
-        <v>741000</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B25" s="11" t="s">
+      <c r="F24" s="28">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B25" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="29">
+        <f>C2*C3*C4</f>
+        <v>2875000</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B26" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="29">
+        <f>SUM(F27:F30)</f>
+        <v>1081860</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B27" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="17">
+      <c r="C27" s="15">
         <v>12</v>
       </c>
-      <c r="D25" s="18">
+      <c r="D27" s="16">
         <v>6500</v>
       </c>
-      <c r="E25" s="24" t="s">
+      <c r="E27" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F27" s="30">
+        <f>(D27*C27)*1.46*C6</f>
+        <v>341640</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B28" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="34">
-        <v>78000</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B26" s="11" t="s">
+      <c r="C28" s="15">
+        <v>6</v>
+      </c>
+      <c r="D28" s="16">
+        <v>4000</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F28" s="30">
+        <f>(D28*C28)*1.46*C6</f>
+        <v>105120</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B29" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="17">
-        <v>6</v>
-      </c>
-      <c r="D26" s="18">
+      <c r="C29" s="15">
+        <v>25</v>
+      </c>
+      <c r="D29" s="16">
         <v>4000</v>
       </c>
-      <c r="E26" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="F26" s="34">
-        <v>24000</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B27" s="11" t="s">
+      <c r="E29" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F29" s="30">
+        <f>(D29*C29)*1.46*C6</f>
+        <v>438000</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B30" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="17">
+      <c r="C30" s="15">
+        <v>10</v>
+      </c>
+      <c r="D30" s="16">
+        <v>4500</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" s="30">
+        <f>(D30*C30)*1.46*C6</f>
+        <v>197100</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B31" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="15"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="29">
+        <f>SUM(F32:F35)</f>
+        <v>224468.08510638302</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B32" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" s="15">
+        <v>1</v>
+      </c>
+      <c r="D32" s="16">
+        <v>4000</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="30">
+        <f>(D32*C32*13)/0.94</f>
+        <v>55319.148936170219</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B33" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C33" s="17">
+        <v>4</v>
+      </c>
+      <c r="D33" s="16">
+        <v>2000</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" s="30">
+        <f>(D33*C33*5*C6)/0.94</f>
+        <v>127659.57446808512</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B34" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" s="17">
+        <v>1</v>
+      </c>
+      <c r="D34" s="16">
+        <v>5000</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="30">
+        <f>((D34*C34)*3)/0.94</f>
+        <v>15957.44680851064</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B35" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D27" s="18">
-        <v>4000</v>
-      </c>
-      <c r="E27" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="F27" s="34">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B28" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="17">
-        <v>10</v>
-      </c>
-      <c r="D28" s="18">
-        <v>4500</v>
-      </c>
-      <c r="E28" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="F28" s="34">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B29" s="27" t="s">
+      <c r="C35" s="17">
+        <v>2</v>
+      </c>
+      <c r="D35" s="16">
+        <v>2000</v>
+      </c>
+      <c r="E35" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="31"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="30">
-        <f>SUM(F30:F33)</f>
-        <v>224468.08617021277</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B30" s="11" t="s">
+      <c r="F35" s="30">
+        <f>((C35*D35)*6)/0.94</f>
+        <v>25531.914893617024</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B36" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="29">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B37" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="9"/>
+      <c r="D37" s="16">
+        <v>280000</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F37" s="29">
+        <f>D37*C6</f>
+        <v>840000</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B38" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="29">
+        <f>F39</f>
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B39" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="C39" s="15">
+        <v>3</v>
+      </c>
+      <c r="D39" s="10">
+        <v>220000</v>
+      </c>
+      <c r="E39" s="9"/>
+      <c r="F39" s="29">
+        <f>D39</f>
+        <v>220000</v>
+      </c>
+      <c r="G39" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B40" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="33">
-        <v>55319.15</v>
-      </c>
-    </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B31" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C31" s="19">
-        <v>4</v>
-      </c>
-      <c r="D31" s="18">
-        <v>2000</v>
-      </c>
-      <c r="E31" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="F31" s="33">
-        <f>((D31*C31)*5*C5)/0.94</f>
-        <v>127659.57446808512</v>
-      </c>
-      <c r="G31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B32" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C32" s="19">
-        <v>1</v>
-      </c>
-      <c r="D32" s="18">
-        <v>5000</v>
-      </c>
-      <c r="E32" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="F32" s="33">
-        <f>((C32*D32)*3)/0.94</f>
-        <v>15957.44680851064</v>
-      </c>
-      <c r="G32" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B33" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C33" s="19">
-        <v>2</v>
-      </c>
-      <c r="D33" s="18">
-        <v>2000</v>
-      </c>
-      <c r="E33" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="F33" s="33">
-        <f>(D33*C33)*6/0.94</f>
-        <v>25531.914893617024</v>
-      </c>
-      <c r="G33" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B34" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="35">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B35" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="35">
-        <v>840000</v>
-      </c>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B36" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C36" s="27"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="27"/>
-      <c r="F36" s="35">
-        <f>150000*C5</f>
-        <v>450000</v>
-      </c>
-    </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B37" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="35">
-        <f>C6*C5</f>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="29">
+        <f>C8*C6</f>
         <v>60000</v>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="F39" s="20"/>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F42" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>